<commit_message>
HTML + timetable updates (common)
</commit_message>
<xml_diff>
--- a/dummy-input.xlsx
+++ b/dummy-input.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
   <si>
     <t>Parámetro</t>
   </si>
@@ -29,10 +29,16 @@
     <t>Nº equipos de Professional</t>
   </si>
   <si>
+    <t>Nº de equipos que se clasifican</t>
+  </si>
+  <si>
     <t>Nº de Jueces para el portfolio técnico</t>
   </si>
   <si>
     <t>Nº de Jueces para el portfolio de empresa</t>
+  </si>
+  <si>
+    <t>Nº de Jueces para el escrutinio</t>
   </si>
   <si>
     <t>Nº de Jueces para la presentación verbal</t>
@@ -524,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -564,7 +570,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -580,7 +586,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -588,7 +594,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -604,7 +610,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -612,7 +618,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -620,23 +626,23 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="1">
-        <v>45825.58333333333</v>
+      <c r="B13">
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="1">
-        <v>45825.58333333333</v>
+      <c r="B14">
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -644,7 +650,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="1">
-        <v>45825.711805555555</v>
+        <v>45825.58333333333</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -652,7 +658,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="1">
-        <v>45826.29166666667</v>
+        <v>45825.58333333333</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -660,7 +666,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="1">
-        <v>45826.29166666667</v>
+        <v>45825.711805555555</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -668,7 +674,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="1">
-        <v>45826.66666666667</v>
+        <v>45826.29166666667</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -676,7 +682,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="1">
-        <v>45827.29166666667</v>
+        <v>45826.29166666667</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -684,7 +690,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="1">
-        <v>45827.29166666667</v>
+        <v>45826.66666666667</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -692,6 +698,22 @@
         <v>21</v>
       </c>
       <c r="B21" s="1">
+        <v>45827.29166666667</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45827.29166666667</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="1">
         <v>45827.5</v>
       </c>
     </row>
@@ -708,13 +730,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -722,10 +744,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -733,10 +755,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -744,10 +766,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
         <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -755,10 +777,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -766,10 +788,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -777,10 +799,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -788,10 +810,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -799,10 +821,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -810,10 +832,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -821,10 +843,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -832,10 +854,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -843,10 +865,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -854,10 +876,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
         <v>40</v>
-      </c>
-      <c r="C14" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -865,10 +887,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -876,10 +898,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -887,10 +909,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -898,10 +920,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Readme + Input + Table
</commit_message>
<xml_diff>
--- a/dummy-input.xlsx
+++ b/dummy-input.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="81">
   <si>
     <t>Parámetro</t>
   </si>
@@ -56,16 +56,43 @@
     <t>Carreras Professional</t>
   </si>
   <si>
-    <t>StartDate</t>
+    <t>NumberOfDays</t>
+  </si>
+  <si>
+    <t>Dia 1 Start</t>
   </si>
   <si>
     <t>2025-06-17T07:00:00.000Z</t>
   </si>
   <si>
-    <t>EndDate</t>
-  </si>
-  <si>
-    <t>2025-06-17T17:00:00.000Z</t>
+    <t>Dia 1 End</t>
+  </si>
+  <si>
+    <t>2025-06-17T12:00:00.000Z</t>
+  </si>
+  <si>
+    <t>Dia 2 Start</t>
+  </si>
+  <si>
+    <t>2025-06-18T07:00:00.000Z</t>
+  </si>
+  <si>
+    <t>Dia 2 End</t>
+  </si>
+  <si>
+    <t>2025-06-18T10:00:00.000Z</t>
+  </si>
+  <si>
+    <t>Dia 3 Start</t>
+  </si>
+  <si>
+    <t>2025-06-19T07:00:00.000Z</t>
+  </si>
+  <si>
+    <t>Dia 3 End</t>
+  </si>
+  <si>
+    <t>2025-06-19T17:00:00.000Z</t>
   </si>
   <si>
     <t>Duración registro</t>
@@ -107,7 +134,19 @@
     <t>Duración Presentación Verbal Entry</t>
   </si>
   <si>
+    <t>Duración Presentación Verbal Development</t>
+  </si>
+  <si>
+    <t>Duración Presentación Verbal Professional</t>
+  </si>
+  <si>
     <t>Duración Ceremonia de Clausura y Premios</t>
+  </si>
+  <si>
+    <t>Duración Carrera</t>
+  </si>
+  <si>
+    <t>Tiempo Eliminatorias</t>
   </si>
   <si>
     <t>ID</t>
@@ -592,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -703,85 +742,85 @@
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
-        <v>15</v>
+      <c r="B14">
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
         <v>16</v>
-      </c>
-      <c r="B15" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
         <v>18</v>
-      </c>
-      <c r="B16">
-        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
-      <c r="B17">
-        <v>30</v>
+      <c r="B17" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18">
-        <v>60</v>
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B21">
-        <v>25</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B22">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B23">
-        <v>15</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B24">
         <v>15</v>
@@ -789,39 +828,39 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B26">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B27">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B28">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B29">
         <v>15</v>
@@ -829,18 +868,74 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B30">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B31">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36">
         <v>60</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -856,13 +951,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -870,10 +965,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -881,10 +976,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -892,10 +987,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -903,10 +998,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -914,10 +1009,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -925,10 +1020,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -936,10 +1031,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -947,10 +1042,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -958,10 +1053,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -969,10 +1064,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -980,10 +1075,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -991,10 +1086,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1002,10 +1097,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1013,10 +1108,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1024,10 +1119,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1035,10 +1130,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1046,10 +1141,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="C18" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1057,10 +1152,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1068,10 +1163,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1079,10 +1174,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1090,10 +1185,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1101,10 +1196,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1112,10 +1207,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1123,10 +1218,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C25" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1134,10 +1229,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1145,10 +1240,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1156,10 +1251,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1167,10 +1262,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C29" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1178,10 +1273,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C30" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1189,10 +1284,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C31" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>